<commit_message>
feat: land SoftCollision surround slots, wire MassMoveScheduler, and PushMap polish
Complete mass soft-collision issues (service, gap slots, scheduler wire, perf checks), update SPECs/configs, and polish PushMap stage advance/agent wiring.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_躯体外观配置表_Manufacture_BodyAppearanceConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_躯体外观配置表_Manufacture_BodyAppearanceConfig.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work\Cursor\Gravedigger2026\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\CursorGame_Git\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
+    <workbookView windowWidth="28800" windowHeight="12280"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="62">
   <si>
     <t>外观ID</t>
   </si>
@@ -230,14 +230,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -693,148 +686,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1187,9 +1180,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="5"/>
   <cols>
-    <col min="4" max="4" width="19.25" customWidth="1"/>
+    <col min="4" max="4" width="19.2545454545455" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1269,9 +1262,6 @@
       <c r="E4" t="s">
         <v>22</v>
       </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
@@ -1309,9 +1299,6 @@
       <c r="E6" t="s">
         <v>31</v>
       </c>
-      <c r="F6" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
@@ -1329,9 +1316,6 @@
       <c r="E7" t="s">
         <v>36</v>
       </c>
-      <c r="F7" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
@@ -1349,9 +1333,6 @@
       <c r="E8" t="s">
         <v>40</v>
       </c>
-      <c r="F8" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
@@ -1369,9 +1350,6 @@
       <c r="E9" t="s">
         <v>44</v>
       </c>
-      <c r="F9" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
@@ -1389,9 +1367,6 @@
       <c r="E10" t="s">
         <v>48</v>
       </c>
-      <c r="F10" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
@@ -1409,9 +1384,6 @@
       <c r="E11" t="s">
         <v>53</v>
       </c>
-      <c r="F11" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
@@ -1428,9 +1400,6 @@
       </c>
       <c r="E12" t="s">
         <v>57</v>
-      </c>
-      <c r="F12" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:6">

</xml_diff>